<commit_message>
Feature: Added new factors relating to treasury yields.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{093A088A-758D-49ED-86EC-4606A17FEC60}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17821072-B212-4262-ABF1-66B484013B0B}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="120" yWindow="2450" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
   <si>
     <t>Fund</t>
   </si>
@@ -78,14 +78,34 @@
   </si>
   <si>
     <t>NEA</t>
+  </si>
+  <si>
+    <t>10 chg4</t>
+  </si>
+  <si>
+    <t>2 chg4</t>
+  </si>
+  <si>
+    <t>curve chg4</t>
+  </si>
+  <si>
+    <t>delta yield 10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -113,21 +133,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -143,6 +167,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -462,58 +490,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.7265625" style="1"/>
+    <col min="10" max="10" width="9.54296875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>50</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>1.6E-2</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>0.16</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>-2.2499999999999999E-2</v>
       </c>
       <c r="F2" s="1">
@@ -522,30 +565,33 @@
       <c r="G2">
         <v>2</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2">
         <v>12</v>
       </c>
-      <c r="I2" s="5">
+      <c r="M2" s="3">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="J2" s="5">
+      <c r="N2" s="3">
         <v>5.1799999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1">
         <v>-2.2499999999999999E-2</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -554,316 +600,479 @@
       <c r="G3">
         <v>2</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3">
         <v>15</v>
       </c>
-      <c r="I3" s="5">
+      <c r="M3" s="3">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="J3" s="5">
+      <c r="N3" s="3">
         <v>6.0600000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2">
-        <v>3</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="D5" s="2">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="E5" s="2">
-        <v>-1.7999999999999999E-2</v>
-      </c>
-      <c r="F5" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="G5" s="1">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1">
+        <v>-2.2499999999999999E-2</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4">
         <v>2</v>
       </c>
-      <c r="H5" s="1">
-        <v>11</v>
-      </c>
-      <c r="I5" s="5">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="J5" s="5">
-        <v>5.6599999999999998E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H4" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <v>27</v>
+      </c>
+      <c r="M4" s="3">
+        <v>4.9000000000000002E-2</v>
+      </c>
+      <c r="N4" s="7">
+        <v>6.83E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>10</v>
+      <c r="F6" s="1">
+        <v>4.2</v>
       </c>
       <c r="G6" s="1">
         <v>2</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="4"/>
+      <c r="I6" s="4"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="1">
         <v>11</v>
       </c>
-      <c r="I6" s="5">
+      <c r="M6" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="J6" s="5">
+      <c r="N6" s="3">
+        <v>5.6599999999999998E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="D7" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E7" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="1">
+        <v>11</v>
+      </c>
+      <c r="M7" s="3">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="N7" s="3">
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="2">
-        <v>32</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="E8" s="2">
-        <v>-0.11</v>
-      </c>
-      <c r="F8" s="1">
-        <v>7</v>
+        <v>12</v>
+      </c>
+      <c r="B8" s="1">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="D8" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E8" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="G8" s="1">
         <v>2</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J8" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L8" s="1">
+        <v>12</v>
+      </c>
+      <c r="M8" s="3">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="N8" s="7">
+        <v>6.3700000000000007E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+      <c r="K9" s="4"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1">
+        <v>32</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-0.11</v>
+      </c>
+      <c r="F10" s="1">
+        <v>7</v>
+      </c>
+      <c r="G10" s="1">
+        <v>2</v>
+      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="1">
         <v>20</v>
       </c>
-      <c r="I8" s="5">
+      <c r="M10" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="J8" s="5">
+      <c r="N10" s="3">
         <v>3.9300000000000002E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B11" s="1">
         <v>32</v>
       </c>
-      <c r="C9" s="2">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="1">
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" s="1">
         <v>2</v>
       </c>
-      <c r="H9" s="1">
-        <v>16</v>
-      </c>
-      <c r="I9" s="5">
+      <c r="H11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J11" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="6">
+        <v>10</v>
+      </c>
+      <c r="M11" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="J9" s="5">
-        <v>5.16E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="J25" s="5"/>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="J27" s="5"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="J28" s="5"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D30" s="2"/>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D32" s="2"/>
+      <c r="N11" s="7">
+        <v>6.3799999999999996E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="N27" s="3"/>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="N28" s="3"/>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="N29" s="3"/>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="N30" s="3"/>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D32" s="1"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D33" s="2"/>
+      <c r="D33" s="1"/>
+    </row>
+    <row r="34" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D35" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Feature: Now able to add and remove securities and update historical data.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17821072-B212-4262-ABF1-66B484013B0B}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C7D8717-B44A-4B92-91F5-DC691B97D325}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="2450" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="19">
   <si>
     <t>Fund</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>delta yield 10</t>
+  </si>
+  <si>
+    <t>updated data</t>
   </si>
 </sst>
 </file>
@@ -490,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -499,7 +502,7 @@
     <col min="11" max="11" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -543,7 +546,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -578,7 +581,7 @@
         <v>5.1799999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -613,7 +616,7 @@
         <v>6.0600000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -657,53 +660,65 @@
         <v>6.83E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1">
-        <v>3</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="E6" s="1">
-        <v>-1.7999999999999999E-2</v>
-      </c>
-      <c r="F6" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="G6" s="1">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1">
+        <v>-2.2499999999999999E-2</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5">
         <v>2</v>
       </c>
+      <c r="H5" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5">
+        <v>27</v>
+      </c>
+      <c r="M5" s="3">
+        <v>4.82E-2</v>
+      </c>
+      <c r="N5" s="7">
+        <v>6.7199999999999996E-2</v>
+      </c>
+      <c r="O5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="1">
-        <v>11</v>
-      </c>
-      <c r="M6" s="3">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="N6" s="3">
-        <v>5.6599999999999998E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -719,8 +734,8 @@
       <c r="E7" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>10</v>
+      <c r="F7" s="1">
+        <v>4.2</v>
       </c>
       <c r="G7" s="1">
         <v>2</v>
@@ -735,10 +750,10 @@
         <v>1.7399999999999999E-2</v>
       </c>
       <c r="N7" s="3">
-        <v>5.91E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+        <v>5.6599999999999998E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -760,130 +775,154 @@
       <c r="G8" s="1">
         <v>2</v>
       </c>
-      <c r="H8" s="4">
-        <v>0.11</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="5">
-        <v>0.36</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>10</v>
-      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="K8" s="4"/>
       <c r="L8" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M8" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="3">
+        <v>5.91E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="D9" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1">
+        <v>2</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="1">
+        <v>12</v>
+      </c>
+      <c r="M9" s="3">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="N9" s="7">
         <v>6.3700000000000007E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1">
-        <v>32</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="E10" s="1">
-        <v>-0.11</v>
-      </c>
-      <c r="F10" s="1">
-        <v>7</v>
-      </c>
-      <c r="G10" s="1">
-        <v>2</v>
-      </c>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="K10" s="4"/>
-      <c r="L10" s="1">
-        <v>20</v>
-      </c>
-      <c r="M10" s="3">
-        <v>4.6600000000000003E-2</v>
-      </c>
-      <c r="N10" s="3">
-        <v>3.9300000000000002E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="1">
         <v>32</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>10</v>
+      <c r="C11" s="1">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="E11" s="1">
+        <v>-0.11</v>
+      </c>
+      <c r="F11" s="1">
+        <v>7</v>
       </c>
       <c r="G11" s="1">
         <v>2</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J11" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L11" s="6">
-        <v>10</v>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="1">
+        <v>20</v>
       </c>
       <c r="M11" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="3">
+        <v>3.9300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1">
+        <v>32</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J12" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L12" s="6">
+        <v>10</v>
+      </c>
+      <c r="M12" s="3">
+        <v>4.6600000000000003E-2</v>
+      </c>
+      <c r="N12" s="7">
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -894,7 +933,7 @@
       <c r="M13" s="3"/>
       <c r="N13" s="3"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -905,7 +944,7 @@
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -916,7 +955,7 @@
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1027,6 +1066,7 @@
       <c r="N25" s="3"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -1040,6 +1080,10 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.35">
@@ -1049,6 +1093,7 @@
       <c r="N28" s="3"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="N29" s="3"/>
@@ -1061,9 +1106,11 @@
     <row r="31" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
+      <c r="N31" s="3"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>
@@ -1073,6 +1120,9 @@
     </row>
     <row r="35" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
+    </row>
+    <row r="36" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D36" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Feature: Change product name and optimizer tab name
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C7D8717-B44A-4B92-91F5-DC691B97D325}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D67A41D0-1709-4E1A-B84A-08FA5B6F2D44}"/>
   <bookViews>
     <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="19">
   <si>
     <t>Fund</t>
   </si>
@@ -92,7 +92,7 @@
     <t>delta yield 10</t>
   </si>
   <si>
-    <t>updated data</t>
+    <t>updated data as of 3/6/26</t>
   </si>
 </sst>
 </file>
@@ -493,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -833,50 +833,62 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="D10" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="1">
+        <v>2</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="1">
+        <v>12</v>
+      </c>
+      <c r="M10" s="3">
+        <v>1.67E-2</v>
+      </c>
+      <c r="N10" s="7">
+        <v>6.3600000000000004E-2</v>
+      </c>
+      <c r="O10" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1">
-        <v>32</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="E11" s="1">
-        <v>-0.11</v>
-      </c>
-      <c r="F11" s="1">
-        <v>7</v>
-      </c>
-      <c r="G11" s="1">
-        <v>2</v>
-      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="K11" s="4"/>
-      <c r="L11" s="1">
-        <v>20</v>
-      </c>
-      <c r="M11" s="3">
-        <v>4.6600000000000003E-2</v>
-      </c>
-      <c r="N11" s="3">
-        <v>3.9300000000000002E-2</v>
-      </c>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -885,64 +897,124 @@
       <c r="B12" s="1">
         <v>32</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>10</v>
+      <c r="C12" s="1">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="E12" s="1">
+        <v>-0.11</v>
+      </c>
+      <c r="F12" s="1">
+        <v>7</v>
       </c>
       <c r="G12" s="1">
         <v>2</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J12" s="5">
-        <v>0.3</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L12" s="6">
-        <v>10</v>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="1">
+        <v>20</v>
       </c>
       <c r="M12" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="3">
+        <v>3.9300000000000002E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1">
+        <v>32</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="1">
+        <v>2</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J13" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="6">
+        <v>10</v>
+      </c>
+      <c r="M13" s="3">
+        <v>4.6600000000000003E-2</v>
+      </c>
+      <c r="N13" s="7">
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-    </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>32</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="5">
+        <v>0.3</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L14" s="6">
+        <v>10</v>
+      </c>
+      <c r="M14" s="3">
+        <v>4.6100000000000002E-2</v>
+      </c>
+      <c r="N14" s="7">
+        <v>6.3299999999999995E-2</v>
+      </c>
+      <c r="O14" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
@@ -1077,6 +1149,7 @@
       <c r="N26" s="3"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -1090,6 +1163,10 @@
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="M28" s="3"/>
       <c r="N28" s="3"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.35">
@@ -1099,6 +1176,7 @@
       <c r="N29" s="3"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="N30" s="3"/>
@@ -1111,18 +1189,23 @@
     <row r="32" spans="2:14" x14ac:dyDescent="0.35">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="N32" s="3"/>
+    </row>
+    <row r="33" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>
-    </row>
-    <row r="34" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D34" s="1"/>
     </row>
-    <row r="35" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
     </row>
-    <row r="36" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D36" s="1"/>
+    </row>
+    <row r="37" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="D37" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bug Fix: Values were not updating immediately in Current Signal when settings changed.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="133" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D67A41D0-1709-4E1A-B84A-08FA5B6F2D44}"/>
+  <xr:revisionPtr revIDLastSave="158" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3C1112-8A63-4E47-82FB-41BE9C010086}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="20">
   <si>
     <t>Fund</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>updated data as of 3/6/26</t>
+  </si>
+  <si>
+    <t>CLOI</t>
   </si>
 </sst>
 </file>
@@ -136,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -155,6 +158,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,7 +505,7 @@
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="8.7265625" style="1"/>
     <col min="10" max="10" width="9.54296875" style="5" customWidth="1"/>
-    <col min="11" max="11" width="11.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.36328125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -533,7 +539,7 @@
       <c r="J1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="8" t="s">
         <v>17</v>
       </c>
       <c r="L1" s="2" t="s">
@@ -570,7 +576,6 @@
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
-      <c r="K2" s="4"/>
       <c r="L2">
         <v>12</v>
       </c>
@@ -605,7 +610,6 @@
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="K3" s="4"/>
       <c r="L3">
         <v>15</v>
       </c>
@@ -647,7 +651,7 @@
       <c r="J4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L4">
@@ -691,7 +695,7 @@
       <c r="J5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L5">
@@ -714,7 +718,6 @@
       <c r="E6" s="1"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="K6" s="4"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
     </row>
@@ -742,7 +745,6 @@
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="K7" s="4"/>
       <c r="L7" s="1">
         <v>11</v>
       </c>
@@ -777,7 +779,6 @@
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="K8" s="4"/>
       <c r="L8" s="1">
         <v>11</v>
       </c>
@@ -819,7 +820,7 @@
       <c r="J9" s="5">
         <v>0.36</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L9" s="1">
@@ -863,7 +864,7 @@
       <c r="J10" s="5">
         <v>0.36</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L10" s="1">
@@ -886,7 +887,6 @@
       <c r="E11" s="1"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="K11" s="4"/>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
     </row>
@@ -914,7 +914,6 @@
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
-      <c r="K12" s="4"/>
       <c r="L12" s="1">
         <v>20</v>
       </c>
@@ -956,7 +955,7 @@
       <c r="J13" s="5">
         <v>0.3</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L13" s="6">
@@ -1000,7 +999,7 @@
       <c r="J14" s="5">
         <v>0.3</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="8" t="s">
         <v>10</v>
       </c>
       <c r="L14" s="6">
@@ -1023,20 +1022,55 @@
       <c r="E15" s="1"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-      <c r="K15" s="4"/>
       <c r="M15" s="3"/>
       <c r="N15" s="3"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K16" s="8">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>7</v>
+      </c>
+      <c r="M16" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="N16" s="7">
+        <v>0.08</v>
+      </c>
+      <c r="O16" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B17" s="1"/>
@@ -1045,7 +1079,6 @@
       <c r="E17" s="1"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
-      <c r="K17" s="4"/>
       <c r="M17" s="3"/>
       <c r="N17" s="3"/>
     </row>
@@ -1056,7 +1089,6 @@
       <c r="E18" s="1"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-      <c r="K18" s="4"/>
       <c r="M18" s="3"/>
       <c r="N18" s="3"/>
     </row>
@@ -1067,7 +1099,6 @@
       <c r="E19" s="1"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="K19" s="4"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
     </row>
@@ -1078,7 +1109,6 @@
       <c r="E20" s="1"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="K20" s="4"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
     </row>
@@ -1089,7 +1119,6 @@
       <c r="E21" s="1"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
-      <c r="K21" s="4"/>
       <c r="M21" s="3"/>
       <c r="N21" s="3"/>
     </row>
@@ -1100,7 +1129,6 @@
       <c r="E22" s="1"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="K22" s="4"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
     </row>
@@ -1111,7 +1139,6 @@
       <c r="E23" s="1"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="K23" s="4"/>
       <c r="M23" s="3"/>
       <c r="N23" s="3"/>
     </row>
@@ -1122,7 +1149,6 @@
       <c r="E24" s="1"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="K24" s="4"/>
       <c r="M24" s="3"/>
       <c r="N24" s="3"/>
     </row>
@@ -1133,7 +1159,6 @@
       <c r="E25" s="1"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="K25" s="4"/>
       <c r="M25" s="3"/>
       <c r="N25" s="3"/>
     </row>
@@ -1144,7 +1169,6 @@
       <c r="E26" s="1"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="K26" s="4"/>
       <c r="M26" s="3"/>
       <c r="N26" s="3"/>
     </row>
@@ -1155,7 +1179,6 @@
       <c r="E27" s="1"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="K27" s="4"/>
       <c r="M27" s="3"/>
       <c r="N27" s="3"/>
     </row>
@@ -1165,7 +1188,6 @@
       <c r="E28" s="1"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="K28" s="4"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
     </row>

</xml_diff>

<commit_message>
Enahncement: Fine tuned CLOI parameters and added JMST
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="158" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3C1112-8A63-4E47-82FB-41BE9C010086}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69653523-E6B4-4EBA-95A0-9200AF59CEB7}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="830" yWindow="4450" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="23">
   <si>
     <t>Fund</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t>CLOI</t>
+  </si>
+  <si>
+    <t>Cash Rate</t>
+  </si>
+  <si>
+    <t>JMST</t>
+  </si>
+  <si>
+    <t>data as of 3/6/26</t>
   </si>
 </sst>
 </file>
@@ -139,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -161,6 +170,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,16 +515,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="8.7265625" style="1"/>
     <col min="10" max="10" width="9.54296875" style="5" customWidth="1"/>
     <col min="11" max="11" width="11.36328125" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -545,14 +562,17 @@
       <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -580,13 +600,16 @@
         <v>12</v>
       </c>
       <c r="M2" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="N2" s="3">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
         <v>5.1799999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -614,13 +637,16 @@
         <v>15</v>
       </c>
       <c r="M3" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="N3" s="3">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="N3" s="3">
+      <c r="O3" s="3">
         <v>6.0600000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -658,13 +684,16 @@
         <v>27</v>
       </c>
       <c r="M4" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="N4" s="3">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="N4" s="7">
+      <c r="O4" s="7">
         <v>6.83E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -702,26 +731,29 @@
         <v>27</v>
       </c>
       <c r="M5" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="N5" s="3">
         <v>4.82E-2</v>
       </c>
-      <c r="N5" s="7">
+      <c r="O5" s="7">
         <v>6.7199999999999996E-2</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
-      <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -748,14 +780,17 @@
       <c r="L7" s="1">
         <v>11</v>
       </c>
-      <c r="M7" s="3">
+      <c r="M7" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="N7" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="N7" s="3">
+      <c r="O7" s="3">
         <v>5.6599999999999998E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -782,14 +817,17 @@
       <c r="L8" s="1">
         <v>11</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="N8" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="N8" s="3">
+      <c r="O8" s="3">
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -826,14 +864,17 @@
       <c r="L9" s="1">
         <v>12</v>
       </c>
-      <c r="M9" s="3">
+      <c r="M9" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="N9" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="N9" s="7">
+      <c r="O9" s="7">
         <v>6.3700000000000007E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -870,27 +911,30 @@
       <c r="L10" s="1">
         <v>12</v>
       </c>
-      <c r="M10" s="3">
+      <c r="M10" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="N10" s="3">
         <v>1.67E-2</v>
       </c>
-      <c r="N10" s="7">
+      <c r="O10" s="7">
         <v>6.3600000000000004E-2</v>
       </c>
-      <c r="O10" t="s">
+      <c r="P10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
-      <c r="M11" s="3"/>
       <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -917,14 +961,17 @@
       <c r="L12" s="1">
         <v>20</v>
       </c>
-      <c r="M12" s="3">
+      <c r="M12" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="N12" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="N12" s="3">
+      <c r="O12" s="3">
         <v>3.9300000000000002E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -961,14 +1008,17 @@
       <c r="L13" s="6">
         <v>10</v>
       </c>
-      <c r="M13" s="3">
+      <c r="M13" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="N13" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="N13" s="7">
+      <c r="O13" s="7">
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1005,27 +1055,30 @@
       <c r="L14" s="6">
         <v>10</v>
       </c>
-      <c r="M14" s="3">
+      <c r="M14" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="N14" s="3">
         <v>4.6100000000000002E-2</v>
       </c>
-      <c r="N14" s="7">
+      <c r="O14" s="7">
         <v>6.3299999999999995E-2</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
-      <c r="M15" s="3"/>
       <c r="N15" s="3"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="O15" s="3"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1063,155 +1116,318 @@
         <v>7</v>
       </c>
       <c r="M16" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="N16" s="3">
         <v>7.1599999999999997E-2</v>
       </c>
-      <c r="N16" s="7">
+      <c r="O16" s="7">
         <v>0.08</v>
       </c>
-      <c r="O16" t="s">
+      <c r="P16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K17" s="8">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>7</v>
+      </c>
+      <c r="M17" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="N17" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="O17" s="7">
+        <v>7.9299999999999995E-2</v>
+      </c>
+      <c r="P17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K18" s="8">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <v>7</v>
+      </c>
+      <c r="M18" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="N18" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="O18" s="7">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="P18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="M19" s="3"/>
       <c r="N19" s="3"/>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-    </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O19" s="3"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="1">
+        <v>2</v>
+      </c>
+      <c r="C20" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="I20" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K20" s="8">
+        <v>1</v>
+      </c>
+      <c r="L20">
+        <v>10</v>
+      </c>
+      <c r="M20" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="N20" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="O20" s="7">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="P20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1">
+        <v>2</v>
+      </c>
+      <c r="C21" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="I21" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21" s="11">
+        <v>8</v>
+      </c>
+      <c r="M21" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="N21" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="O21" s="7">
+        <v>2.75E-2</v>
+      </c>
+      <c r="P21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="M22" s="3"/>
       <c r="N22" s="3"/>
-    </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="M23" s="3"/>
       <c r="N23" s="3"/>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="M24" s="3"/>
       <c r="N24" s="3"/>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="M25" s="3"/>
       <c r="N25" s="3"/>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O25" s="3"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="M26" s="3"/>
       <c r="N26" s="3"/>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O26" s="3"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="M27" s="3"/>
       <c r="N27" s="3"/>
-    </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O27" s="3"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="M28" s="3"/>
       <c r="N28" s="3"/>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O28" s="3"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
-      <c r="N29" s="3"/>
-    </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O29" s="3"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
-      <c r="N30" s="3"/>
-    </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O30" s="3"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
-      <c r="N31" s="3"/>
-    </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="O31" s="3"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
-      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
     </row>
     <row r="33" spans="4:5" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>

</xml_diff>

<commit_message>
Enhancement: Don't jump out of current tab when changing security
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69653523-E6B4-4EBA-95A0-9200AF59CEB7}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{714B0CD5-896D-4F36-BC03-D814065C12FF}"/>
   <bookViews>
-    <workbookView xWindow="830" yWindow="4450" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -148,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -177,6 +177,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1235,6 +1236,7 @@
       <c r="E19" s="1"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
+      <c r="L19" s="11"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
     </row>
@@ -1272,8 +1274,8 @@
       <c r="K20" s="8">
         <v>1</v>
       </c>
-      <c r="L20">
-        <v>10</v>
+      <c r="L20" s="11">
+        <v>8</v>
       </c>
       <c r="M20" s="3">
         <v>2.3E-2</v>
@@ -1322,8 +1324,8 @@
       <c r="K21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L21" s="11">
-        <v>8</v>
+      <c r="L21" s="12">
+        <v>10</v>
       </c>
       <c r="M21" s="3">
         <v>2.3E-2</v>

</xml_diff>

<commit_message>
Configuration: Changed some settings
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{714B0CD5-896D-4F36-BC03-D814065C12FF}"/>
+  <xr:revisionPtr revIDLastSave="231" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6729CBB4-EB5D-4EC5-8BBD-97749C12C6C6}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="2000" yWindow="650" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="25">
   <si>
     <t>Fund</t>
   </si>
@@ -105,6 +105,12 @@
   </si>
   <si>
     <t>data as of 3/6/26</t>
+  </si>
+  <si>
+    <t>INCM</t>
+  </si>
+  <si>
+    <t>data as of 3/11/26</t>
   </si>
 </sst>
 </file>
@@ -148,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -177,7 +183,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1324,7 +1329,7 @@
       <c r="K21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L21" s="12">
+      <c r="L21">
         <v>10</v>
       </c>
       <c r="M21" s="3">
@@ -1351,14 +1356,54 @@
       <c r="O22" s="3"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="E23" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="I23" s="4">
+        <v>7.6999999999999999E-2</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23" s="3">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="N23" s="3">
+        <v>0.1082</v>
+      </c>
+      <c r="O23" s="7">
+        <v>0.14130000000000001</v>
+      </c>
+      <c r="P23" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B24" s="1"/>

</xml_diff>

<commit_message>
Bug Fix: When a date is invalid and the error message pops, remove the message when the date is fixed.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="231" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6729CBB4-EB5D-4EC5-8BBD-97749C12C6C6}"/>
+  <xr:revisionPtr revIDLastSave="251" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4813DE64-A9F4-4A0F-96B0-DCB40DC25F2D}"/>
   <bookViews>
-    <workbookView xWindow="2000" yWindow="650" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="26">
   <si>
     <t>Fund</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>data as of 3/11/26</t>
+  </si>
+  <si>
+    <t>Use drop instead of delta yield 10</t>
   </si>
 </sst>
 </file>
@@ -521,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -1119,7 +1122,7 @@
         <v>1</v>
       </c>
       <c r="L16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M16" s="3">
         <v>0.04</v>
@@ -1169,7 +1172,7 @@
         <v>1</v>
       </c>
       <c r="L17">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M17" s="3">
         <v>3.6499999999999998E-2</v>
@@ -1219,7 +1222,7 @@
         <v>1</v>
       </c>
       <c r="L18">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M18" s="3">
         <v>3.6499999999999998E-2</v>
@@ -1235,65 +1238,65 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="L19" s="11"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19">
+        <v>9</v>
+      </c>
+      <c r="M19" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="N19" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="O19" s="7">
+        <v>8.4900000000000003E-2</v>
+      </c>
+      <c r="P19" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="1">
-        <v>2</v>
-      </c>
-      <c r="C20" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="I20" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="K20" s="8">
-        <v>1</v>
-      </c>
-      <c r="L20" s="11">
-        <v>8</v>
-      </c>
-      <c r="M20" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="N20" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="O20" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="P20" t="s">
-        <v>22</v>
-      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="L20" s="11"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1326,11 +1329,11 @@
       <c r="J21" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K21" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="L21">
-        <v>10</v>
+      <c r="K21" s="8">
+        <v>1</v>
+      </c>
+      <c r="L21" s="11">
+        <v>8</v>
       </c>
       <c r="M21" s="3">
         <v>2.3E-2</v>
@@ -1339,81 +1342,121 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="O21" s="7">
-        <v>2.75E-2</v>
+        <v>2.7099999999999999E-2</v>
       </c>
       <c r="P21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="I22" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L22">
+        <v>10</v>
+      </c>
+      <c r="M22" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="N22" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="O22" s="7">
+        <v>2.75E-2</v>
+      </c>
+      <c r="P22" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="1">
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="1">
         <v>0.125</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E24" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H23" s="4">
+      <c r="F24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H24" s="4">
         <v>0.1</v>
       </c>
-      <c r="I23" s="4">
+      <c r="I24" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="J23" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="K23" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="L23">
-        <v>10</v>
-      </c>
-      <c r="M23" s="3">
+      <c r="J24" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K24" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24">
+        <v>10</v>
+      </c>
+      <c r="M24" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="N23" s="3">
+      <c r="N24" s="3">
         <v>0.1082</v>
       </c>
-      <c r="O23" s="7">
+      <c r="O24" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="P23" t="s">
+      <c r="P24" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B25" s="1"/>
@@ -1446,6 +1489,7 @@
       <c r="O27" s="3"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -1458,6 +1502,9 @@
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="N29" s="3"/>
       <c r="O29" s="3"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.35">
@@ -1467,6 +1514,7 @@
       <c r="O30" s="3"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="O31" s="3"/>
@@ -1476,21 +1524,26 @@
       <c r="E32" s="1"/>
       <c r="O32" s="3"/>
     </row>
-    <row r="33" spans="4:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D34" s="1"/>
-    </row>
-    <row r="35" spans="4:5" x14ac:dyDescent="0.35">
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
     </row>
-    <row r="36" spans="4:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D36" s="1"/>
     </row>
-    <row r="37" spans="4:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="4:15" x14ac:dyDescent="0.35">
+      <c r="D38" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Data: Changed parameters for NEA and spreadsheet data
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="251" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4813DE64-A9F4-4A0F-96B0-DCB40DC25F2D}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5957689D-906B-4D82-8ED9-2B3E73BBFAD5}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="27">
   <si>
     <t>Fund</t>
   </si>
@@ -114,6 +114,9 @@
   </si>
   <si>
     <t>Use drop instead of delta yield 10</t>
+  </si>
+  <si>
+    <t>data as of 3/9/26</t>
   </si>
 </sst>
 </file>
@@ -524,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="6" max="6" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -1017,7 +1020,7 @@
       <c r="L13" s="6">
         <v>10</v>
       </c>
-      <c r="M13" s="10">
+      <c r="M13" s="4">
         <v>0.04</v>
       </c>
       <c r="N13" s="3">
@@ -1064,7 +1067,7 @@
       <c r="L14" s="6">
         <v>10</v>
       </c>
-      <c r="M14" s="10">
+      <c r="M14" s="4">
         <v>0.04</v>
       </c>
       <c r="N14" s="3">
@@ -1078,64 +1081,61 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="5">
+        <v>0.48</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L15" s="6">
+        <v>93</v>
+      </c>
+      <c r="M15" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="N15" s="3">
+        <v>4.6100000000000002E-2</v>
+      </c>
+      <c r="O15" s="7">
+        <v>8.5300000000000001E-2</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="K16" s="8">
-        <v>1</v>
-      </c>
-      <c r="L16">
-        <v>9</v>
-      </c>
-      <c r="M16" s="3">
-        <v>0.04</v>
-      </c>
-      <c r="N16" s="3">
-        <v>7.1599999999999997E-2</v>
-      </c>
-      <c r="O16" s="7">
-        <v>0.08</v>
-      </c>
-      <c r="P16" t="s">
-        <v>18</v>
-      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -1175,13 +1175,13 @@
         <v>9</v>
       </c>
       <c r="M17" s="3">
-        <v>3.6499999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="N17" s="3">
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="O17" s="7">
-        <v>7.9299999999999995E-2</v>
+        <v>0.08</v>
       </c>
       <c r="P17" t="s">
         <v>18</v>
@@ -1209,8 +1209,8 @@
       <c r="G18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H18" s="4">
-        <v>0.1225</v>
+      <c r="H18" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>10</v>
@@ -1231,7 +1231,7 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="O18" s="7">
-        <v>8.0500000000000002E-2</v>
+        <v>7.9299999999999995E-2</v>
       </c>
       <c r="P18" t="s">
         <v>18</v>
@@ -1244,8 +1244,8 @@
       <c r="B19" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="1">
-        <v>0.04</v>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D19" s="1">
         <v>0.1</v>
@@ -1268,8 +1268,8 @@
       <c r="J19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K19" s="8" t="s">
-        <v>10</v>
+      <c r="K19" s="8">
+        <v>1</v>
       </c>
       <c r="L19">
         <v>9</v>
@@ -1281,72 +1281,72 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="O19" s="7">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="P19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L20">
+        <v>9</v>
+      </c>
+      <c r="M20" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="N20" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="O20" s="7">
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="P19" t="s">
+      <c r="P20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="L20" s="11"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-    </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="1">
-        <v>2</v>
-      </c>
-      <c r="C21" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21">
-        <v>2</v>
-      </c>
-      <c r="H21" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="I21" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="8">
-        <v>1</v>
-      </c>
-      <c r="L21" s="11">
-        <v>8</v>
-      </c>
-      <c r="M21" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="N21" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="O21" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="P21" t="s">
-        <v>22</v>
-      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="L21" s="11"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -1379,11 +1379,11 @@
       <c r="J22" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K22" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="L22">
-        <v>10</v>
+      <c r="K22" s="8">
+        <v>1</v>
+      </c>
+      <c r="L22" s="11">
+        <v>8</v>
       </c>
       <c r="M22" s="3">
         <v>2.3E-2</v>
@@ -1392,81 +1392,121 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="O22" s="7">
-        <v>2.75E-2</v>
+        <v>2.7099999999999999E-2</v>
       </c>
       <c r="P22" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="N23" s="3"/>
-      <c r="O23" s="3"/>
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1">
+        <v>2</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L23">
+        <v>10</v>
+      </c>
+      <c r="M23" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="N23" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="O23" s="7">
+        <v>2.7799999999999998E-2</v>
+      </c>
+      <c r="P23" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="1">
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1">
         <v>0.125</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E25" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H24" s="4">
+      <c r="F25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H25" s="4">
         <v>0.1</v>
       </c>
-      <c r="I24" s="4">
+      <c r="I25" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="J24" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="K24" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="L24">
-        <v>10</v>
-      </c>
-      <c r="M24" s="3">
+      <c r="J25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25">
+        <v>10</v>
+      </c>
+      <c r="M25" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="N24" s="3">
+      <c r="N25" s="3">
         <v>0.1082</v>
       </c>
-      <c r="O24" s="7">
+      <c r="O25" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="P24" t="s">
+      <c r="P25" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="N25" s="3"/>
-      <c r="O25" s="3"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B26" s="1"/>
@@ -1499,6 +1539,7 @@
       <c r="O28" s="3"/>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -1511,6 +1552,9 @@
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="N30" s="3"/>
       <c r="O30" s="3"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.35">
@@ -1520,6 +1564,7 @@
       <c r="O31" s="3"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="C32" s="1"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="O32" s="3"/>
@@ -1532,9 +1577,11 @@
     <row r="34" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
+      <c r="O34" s="3"/>
     </row>
     <row r="35" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
     </row>
     <row r="36" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D36" s="1"/>
@@ -1544,6 +1591,9 @@
     </row>
     <row r="38" spans="4:15" x14ac:dyDescent="0.35">
       <c r="D38" s="1"/>
+    </row>
+    <row r="39" spans="4:15" x14ac:dyDescent="0.35">
+      <c r="D39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Enhancement: Better parms for NEA. Updated history files
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="318" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15F3C1A7-89C7-4F3D-8CB3-0518F86D1B35}"/>
+  <xr:revisionPtr revIDLastSave="341" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A977B3F1-8ACC-4A94-A41D-2377F43C6693}"/>
   <bookViews>
-    <workbookView xWindow="500" yWindow="470" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="-1340" yWindow="690" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="33">
   <si>
     <t>Fund</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>BUY SIGNALS</t>
+  </si>
+  <si>
+    <t>updated data as of 3/20/26 discovered during walk forward</t>
   </si>
 </sst>
 </file>
@@ -200,10 +203,10 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -554,10 +557,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1143,75 +1146,75 @@
       <c r="N16" s="6">
         <v>93</v>
       </c>
-      <c r="O16" s="10">
+      <c r="O16" s="11">
         <v>0.04</v>
       </c>
       <c r="P16" s="3">
         <v>4.6100000000000002E-2</v>
       </c>
       <c r="Q16" s="7">
-        <v>8.5300000000000001E-2</v>
+        <v>8.3500000000000005E-2</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J17" s="1">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N17" s="6">
+        <v>80</v>
+      </c>
+      <c r="O17" s="11">
+        <v>0.04</v>
+      </c>
+      <c r="P17" s="3">
+        <v>4.4400000000000002E-2</v>
+      </c>
+      <c r="Q17" s="7">
+        <v>8.5900000000000004E-2</v>
+      </c>
+      <c r="R17" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L18" s="8">
-        <v>1</v>
-      </c>
-      <c r="N18">
-        <v>9</v>
-      </c>
-      <c r="O18" s="3">
-        <v>0.04</v>
-      </c>
-      <c r="P18" s="3">
-        <v>7.1599999999999997E-2</v>
-      </c>
-      <c r="Q18" s="7">
-        <v>0.08</v>
-      </c>
-      <c r="R18" t="s">
-        <v>18</v>
-      </c>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1251,13 +1254,13 @@
         <v>9</v>
       </c>
       <c r="O19" s="3">
-        <v>3.6499999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="P19" s="3">
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q19" s="7">
-        <v>7.9299999999999995E-2</v>
+        <v>0.08</v>
       </c>
       <c r="R19" t="s">
         <v>18</v>
@@ -1276,8 +1279,8 @@
       <c r="D20" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E20" s="4">
-        <v>0.1225</v>
+      <c r="E20" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>10</v>
@@ -1307,7 +1310,7 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q20" s="7">
-        <v>8.0500000000000002E-2</v>
+        <v>7.9299999999999995E-2</v>
       </c>
       <c r="R20" t="s">
         <v>18</v>
@@ -1338,14 +1341,14 @@
       <c r="I21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J21" s="1">
-        <v>0.04</v>
+      <c r="J21" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L21" s="8" t="s">
-        <v>10</v>
+      <c r="L21" s="8">
+        <v>1</v>
       </c>
       <c r="N21">
         <v>9</v>
@@ -1357,72 +1360,72 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q21" s="7">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="R21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J22" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N22">
+        <v>9</v>
+      </c>
+      <c r="O22" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="P22" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="Q22" s="7">
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="R21" t="s">
+      <c r="R22" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="N22" s="11"/>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-    </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E23" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="F23" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I23" s="1">
-        <v>2</v>
-      </c>
-      <c r="J23" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="K23">
-        <v>2</v>
-      </c>
-      <c r="L23" s="8">
-        <v>1</v>
-      </c>
-      <c r="N23" s="11">
-        <v>8</v>
-      </c>
-      <c r="O23" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="P23" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="Q23" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="R23" t="s">
-        <v>22</v>
-      </c>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="N23" s="10"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1455,11 +1458,11 @@
       <c r="K24">
         <v>2</v>
       </c>
-      <c r="L24" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N24">
-        <v>10</v>
+      <c r="L24" s="8">
+        <v>1</v>
+      </c>
+      <c r="N24" s="10">
+        <v>8</v>
       </c>
       <c r="O24" s="3">
         <v>2.3E-2</v>
@@ -1468,141 +1471,181 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="Q24" s="7">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="R24" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I25" s="1">
+        <v>2</v>
+      </c>
+      <c r="J25" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="K25">
+        <v>2</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N25">
+        <v>10</v>
+      </c>
+      <c r="O25" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="P25" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="Q25" s="7">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="R24" t="s">
+      <c r="R25" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="3"/>
-    </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C26" s="1">
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1">
         <v>0.125</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D27" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E27" s="4">
         <v>0.1</v>
       </c>
-      <c r="F26" s="4">
+      <c r="F27" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="G26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N26">
-        <v>10</v>
-      </c>
-      <c r="O26" s="3">
+      <c r="G27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N27">
+        <v>10</v>
+      </c>
+      <c r="O27" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P26" s="3">
+      <c r="P27" s="3">
         <v>0.1082</v>
       </c>
-      <c r="Q26" s="7">
+      <c r="Q27" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="R26" t="s">
+      <c r="R27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-    </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="1">
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1">
         <v>0.22500000000000001</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D29" s="1">
         <v>-1.6E-2</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E29" s="4">
         <v>0.18099999999999999</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K28">
+      <c r="F29" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K29">
         <v>2</v>
       </c>
-      <c r="L28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N28">
+      <c r="L29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N29">
         <v>27</v>
       </c>
-      <c r="O28" s="3">
+      <c r="O29" s="3">
         <v>2.3E-2</v>
       </c>
-      <c r="P28" s="3">
+      <c r="P29" s="3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="Q29" s="7">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="R28" t="s">
+      <c r="R29" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C30" s="1"/>
@@ -1619,6 +1662,7 @@
       <c r="D31" s="1"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
+      <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
@@ -1626,7 +1670,10 @@
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
       <c r="J32" s="1"/>
+      <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
     </row>
     <row r="33" spans="3:17" x14ac:dyDescent="0.35">
@@ -1638,6 +1685,7 @@
     <row r="34" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
+      <c r="J34" s="1"/>
       <c r="Q34" s="3"/>
     </row>
     <row r="35" spans="3:17" x14ac:dyDescent="0.35">
@@ -1648,9 +1696,11 @@
     <row r="36" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
+      <c r="Q36" s="3"/>
     </row>
     <row r="37" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
     </row>
     <row r="38" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C38" s="1"/>
@@ -1660,6 +1710,9 @@
     </row>
     <row r="40" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C40" s="1"/>
+    </row>
+    <row r="41" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="C41" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bug Fix: Fixed some minor issues in walk forward. Optimized SPHY factors
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A977B3F1-8ACC-4A94-A41D-2377F43C6693}"/>
+  <xr:revisionPtr revIDLastSave="362" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F3E96D7-BAC9-463A-86B1-C55864B4D24F}"/>
   <bookViews>
-    <workbookView xWindow="-1340" yWindow="690" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="34">
   <si>
     <t>Fund</t>
   </si>
@@ -135,6 +135,9 @@
   </si>
   <si>
     <t>updated data as of 3/20/26 discovered during walk forward</t>
+  </si>
+  <si>
+    <t>updated data as of 3/20/26</t>
   </si>
 </sst>
 </file>
@@ -178,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -204,9 +207,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,12 +545,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="8.7265625" style="1"/>
     <col min="7" max="8" width="9.54296875" style="5" customWidth="1"/>
+    <col min="11" max="11" width="8.7265625" style="1"/>
     <col min="12" max="12" width="11.36328125" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.36328125" style="8" customWidth="1"/>
     <col min="15" max="15" width="8.7265625" style="3"/>
@@ -593,7 +594,7 @@
       <c r="J2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="L2" s="8" t="s">
@@ -634,7 +635,7 @@
       <c r="J3" s="1">
         <v>1.6E-2</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="1">
         <v>2</v>
       </c>
       <c r="N3">
@@ -671,7 +672,7 @@
       <c r="J4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="1">
         <v>2</v>
       </c>
       <c r="N4">
@@ -715,7 +716,7 @@
       <c r="J5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="1">
         <v>2</v>
       </c>
       <c r="L5" s="8" t="s">
@@ -762,7 +763,7 @@
       <c r="J6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="1">
         <v>2</v>
       </c>
       <c r="L6" s="8" t="s">
@@ -785,58 +786,71 @@
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1">
+        <v>-0.03</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.09</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N7">
+        <v>61</v>
+      </c>
+      <c r="O7" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="P7" s="3">
+        <v>4.7300000000000002E-2</v>
+      </c>
+      <c r="Q7" s="7">
+        <v>7.4099999999999999E-2</v>
+      </c>
+      <c r="R7" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="C8" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="D8" s="1">
-        <v>-1.7999999999999999E-2</v>
-      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="I8" s="1">
-        <v>3</v>
-      </c>
-      <c r="J8" s="1">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="K8" s="1">
-        <v>2</v>
-      </c>
-      <c r="N8" s="1">
-        <v>11</v>
-      </c>
-      <c r="O8" s="4">
-        <v>0.04</v>
-      </c>
-      <c r="P8" s="3">
-        <v>1.7399999999999999E-2</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>5.6599999999999998E-2</v>
-      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>10</v>
+      <c r="B9" s="1">
+        <v>4.2</v>
       </c>
       <c r="C9" s="1">
         <v>7.0000000000000007E-2</v>
@@ -865,7 +879,7 @@
         <v>1.7399999999999999E-2</v>
       </c>
       <c r="Q9" s="3">
-        <v>5.91E-2</v>
+        <v>5.6599999999999998E-2</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
@@ -881,15 +895,8 @@
       <c r="D10" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="E10" s="4">
-        <v>0.11</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0.36</v>
-      </c>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
       <c r="I10" s="1">
         <v>3</v>
       </c>
@@ -899,11 +906,8 @@
       <c r="K10" s="1">
         <v>2</v>
       </c>
-      <c r="L10" s="8" t="s">
-        <v>10</v>
-      </c>
       <c r="N10" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="O10" s="4">
         <v>0.04</v>
@@ -911,8 +915,8 @@
       <c r="P10" s="3">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="Q10" s="7">
-        <v>6.3700000000000007E-2</v>
+      <c r="Q10" s="3">
+        <v>5.91E-2</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
@@ -950,104 +954,104 @@
         <v>10</v>
       </c>
       <c r="N11" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="O11" s="4">
         <v>0.04</v>
       </c>
       <c r="P11" s="3">
+        <v>1.7399999999999999E-2</v>
+      </c>
+      <c r="Q11" s="7">
+        <v>6.3700000000000007E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>-1.7999999999999999E-2</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" s="5">
+        <v>0.36</v>
+      </c>
+      <c r="I12" s="1">
+        <v>3</v>
+      </c>
+      <c r="J12" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="K12" s="1">
+        <v>2</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N12" s="1">
+        <v>14</v>
+      </c>
+      <c r="O12" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="P12" s="3">
         <v>1.54E-2</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="Q12" s="7">
         <v>5.79E-2</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-    </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1">
-        <v>7</v>
-      </c>
-      <c r="C13" s="1">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="D13" s="1">
-        <v>-0.11</v>
-      </c>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="I13" s="1">
-        <v>32</v>
-      </c>
-      <c r="J13" s="1">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="K13" s="1">
-        <v>2</v>
-      </c>
-      <c r="N13" s="1">
-        <v>20</v>
-      </c>
-      <c r="O13" s="4">
-        <v>0.04</v>
-      </c>
-      <c r="P13" s="3">
-        <v>4.6600000000000003E-2</v>
-      </c>
-      <c r="Q13" s="3">
-        <v>3.9300000000000002E-2</v>
-      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0.3</v>
-      </c>
+      <c r="B14" s="1">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="D14" s="1">
+        <v>-0.11</v>
+      </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
       <c r="I14" s="1">
         <v>32</v>
       </c>
-      <c r="J14" s="1" t="s">
-        <v>10</v>
+      <c r="J14" s="1">
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="K14" s="1">
         <v>2</v>
       </c>
-      <c r="L14" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N14" s="6">
-        <v>10</v>
+      <c r="N14" s="1">
+        <v>20</v>
       </c>
       <c r="O14" s="4">
         <v>0.04</v>
@@ -1055,8 +1059,8 @@
       <c r="P14" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="Q14" s="7">
-        <v>6.3799999999999996E-2</v>
+      <c r="Q14" s="3">
+        <v>3.9300000000000002E-2</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
@@ -1100,13 +1104,10 @@
         <v>0.04</v>
       </c>
       <c r="P15" s="3">
-        <v>4.6100000000000002E-2</v>
+        <v>4.6600000000000003E-2</v>
       </c>
       <c r="Q15" s="7">
-        <v>6.3299999999999995E-2</v>
-      </c>
-      <c r="R15" t="s">
-        <v>18</v>
+        <v>6.3799999999999996E-2</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -1116,44 +1117,47 @@
       <c r="B16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="1">
-        <v>0.33</v>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="4">
-        <v>7.0000000000000007E-2</v>
+      <c r="E16" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F16" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="5">
-        <v>0.48</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>10</v>
+        <v>0.3</v>
+      </c>
+      <c r="I16" s="1">
+        <v>32</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>10</v>
+      <c r="K16" s="1">
+        <v>2</v>
       </c>
       <c r="L16" s="8" t="s">
         <v>10</v>
       </c>
       <c r="N16" s="6">
-        <v>93</v>
-      </c>
-      <c r="O16" s="11">
+        <v>10</v>
+      </c>
+      <c r="O16" s="4">
         <v>0.04</v>
       </c>
       <c r="P16" s="3">
         <v>4.6100000000000002E-2</v>
       </c>
       <c r="Q16" s="7">
-        <v>8.3500000000000005E-2</v>
+        <v>6.3299999999999995E-2</v>
+      </c>
+      <c r="R16" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
@@ -1175,96 +1179,93 @@
       <c r="F17" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="5" t="s">
-        <v>10</v>
+      <c r="G17" s="5">
+        <v>0.48</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N17" s="6">
+        <v>93</v>
+      </c>
+      <c r="O17" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="P17" s="3">
+        <v>4.6100000000000002E-2</v>
+      </c>
+      <c r="Q17" s="7">
+        <v>8.3500000000000005E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" s="1">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L17" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N17" s="6">
+      <c r="K18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N18" s="6">
         <v>80</v>
       </c>
-      <c r="O17" s="11">
+      <c r="O18" s="4">
         <v>0.04</v>
       </c>
-      <c r="P17" s="3">
+      <c r="P18" s="3">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="Q17" s="7">
+      <c r="Q18" s="7">
         <v>8.5900000000000004E-2</v>
       </c>
-      <c r="R17" t="s">
+      <c r="R18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-    </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L19" s="8">
-        <v>1</v>
-      </c>
-      <c r="N19">
-        <v>9</v>
-      </c>
-      <c r="O19" s="3">
-        <v>0.04</v>
-      </c>
-      <c r="P19" s="3">
-        <v>7.1599999999999997E-2</v>
-      </c>
-      <c r="Q19" s="7">
-        <v>0.08</v>
-      </c>
-      <c r="R19" t="s">
-        <v>18</v>
-      </c>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -1304,13 +1305,13 @@
         <v>9</v>
       </c>
       <c r="O20" s="3">
-        <v>3.6499999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="P20" s="3">
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q20" s="7">
-        <v>7.9299999999999995E-2</v>
+        <v>0.08</v>
       </c>
       <c r="R20" t="s">
         <v>18</v>
@@ -1329,8 +1330,8 @@
       <c r="D21" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="4">
-        <v>0.1225</v>
+      <c r="E21" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>10</v>
@@ -1360,7 +1361,7 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q21" s="7">
-        <v>8.0500000000000002E-2</v>
+        <v>7.9299999999999995E-2</v>
       </c>
       <c r="R21" t="s">
         <v>18</v>
@@ -1391,14 +1392,14 @@
       <c r="I22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J22" s="1">
-        <v>0.04</v>
+      <c r="J22" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L22" s="8" t="s">
-        <v>10</v>
+      <c r="L22" s="8">
+        <v>1</v>
       </c>
       <c r="N22">
         <v>9</v>
@@ -1410,72 +1411,72 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q22" s="7">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="R22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J23" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N23">
+        <v>9</v>
+      </c>
+      <c r="O23" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="P23" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="Q23" s="7">
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="R22" t="s">
+      <c r="R23" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="N23" s="10"/>
-      <c r="P23" s="3"/>
-      <c r="Q23" s="3"/>
-    </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E24" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="F24" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I24" s="1">
-        <v>2</v>
-      </c>
-      <c r="J24" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="K24">
-        <v>2</v>
-      </c>
-      <c r="L24" s="8">
-        <v>1</v>
-      </c>
-      <c r="N24" s="10">
-        <v>8</v>
-      </c>
-      <c r="O24" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="P24" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="Q24" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="R24" t="s">
-        <v>22</v>
-      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="N24" s="10"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
@@ -1505,14 +1506,14 @@
       <c r="J25" s="1">
         <v>2.4E-2</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="1">
         <v>2</v>
       </c>
-      <c r="L25" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N25">
-        <v>10</v>
+      <c r="L25" s="8">
+        <v>1</v>
+      </c>
+      <c r="N25" s="10">
+        <v>8</v>
       </c>
       <c r="O25" s="3">
         <v>2.3E-2</v>
@@ -1521,141 +1522,181 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="Q25" s="7">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="R25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I26" s="1">
+        <v>2</v>
+      </c>
+      <c r="J26" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="K26" s="1">
+        <v>2</v>
+      </c>
+      <c r="L26" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N26">
+        <v>10</v>
+      </c>
+      <c r="O26" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="P26" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="Q26" s="7">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="R25" t="s">
+      <c r="R26" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-    </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C27" s="1">
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1">
         <v>0.125</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D28" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="E27" s="4">
+      <c r="E28" s="4">
         <v>0.1</v>
       </c>
-      <c r="F27" s="4">
+      <c r="F28" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="G27" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L27" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N27">
-        <v>10</v>
-      </c>
-      <c r="O27" s="3">
+      <c r="G28" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N28">
+        <v>10</v>
+      </c>
+      <c r="O28" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P27" s="3">
+      <c r="P28" s="3">
         <v>0.1082</v>
       </c>
-      <c r="Q27" s="7">
+      <c r="Q28" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="R27" t="s">
+      <c r="R28" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-    </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C29" s="1">
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1">
         <v>0.22500000000000001</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D30" s="1">
         <v>-1.6E-2</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E30" s="4">
         <v>0.18099999999999999</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K29">
+      <c r="F30" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K30" s="1">
         <v>2</v>
       </c>
-      <c r="L29" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N29">
+      <c r="L30" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N30">
         <v>27</v>
       </c>
-      <c r="O29" s="3">
+      <c r="O30" s="3">
         <v>2.3E-2</v>
       </c>
-      <c r="P29" s="3">
+      <c r="P30" s="3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="Q29" s="7">
+      <c r="Q30" s="7">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="R29" t="s">
+      <c r="R30" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="P30" s="3"/>
-      <c r="Q30" s="3"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C31" s="1"/>
@@ -1672,6 +1713,7 @@
       <c r="D32" s="1"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
+      <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
@@ -1679,7 +1721,10 @@
     <row r="33" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
       <c r="J33" s="1"/>
+      <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
     </row>
     <row r="34" spans="3:17" x14ac:dyDescent="0.35">
@@ -1691,6 +1736,7 @@
     <row r="35" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
+      <c r="J35" s="1"/>
       <c r="Q35" s="3"/>
     </row>
     <row r="36" spans="3:17" x14ac:dyDescent="0.35">
@@ -1701,9 +1747,11 @@
     <row r="37" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
+      <c r="Q37" s="3"/>
     </row>
     <row r="38" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
     </row>
     <row r="39" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C39" s="1"/>
@@ -1713,6 +1761,9 @@
     </row>
     <row r="41" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C41" s="1"/>
+    </row>
+    <row r="42" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="C42" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Doc: Updated parameters spreadsheet.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F3E96D7-BAC9-463A-86B1-C55864B4D24F}"/>
+  <xr:revisionPtr revIDLastSave="382" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3D1C113-8AE1-4CAC-8558-9390575B3DD9}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="690" yWindow="1170" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="34">
   <si>
     <t>Fund</t>
   </si>
@@ -545,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -1017,88 +1017,91 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D13" s="1">
+        <v>-1.4E-2</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0.11</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" s="1">
+        <v>5</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K13" s="1">
+        <v>2</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N13" s="1">
+        <v>12</v>
+      </c>
+      <c r="O13" s="4">
+        <v>2.3E-2</v>
+      </c>
+      <c r="P13" s="3">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="Q13" s="7">
+        <v>6.1899999999999997E-2</v>
+      </c>
+      <c r="R13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="1">
-        <v>7</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0.17499999999999999</v>
-      </c>
-      <c r="D14" s="1">
-        <v>-0.11</v>
-      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="I14" s="1">
-        <v>32</v>
-      </c>
-      <c r="J14" s="1">
-        <v>1.4999999999999999E-2</v>
-      </c>
-      <c r="K14" s="1">
-        <v>2</v>
-      </c>
-      <c r="N14" s="1">
-        <v>20</v>
-      </c>
-      <c r="O14" s="4">
-        <v>0.04</v>
-      </c>
-      <c r="P14" s="3">
-        <v>4.6600000000000003E-2</v>
-      </c>
-      <c r="Q14" s="3">
-        <v>3.9300000000000002E-2</v>
-      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0.3</v>
-      </c>
+      <c r="B15" s="1">
+        <v>7</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0.17499999999999999</v>
+      </c>
+      <c r="D15" s="1">
+        <v>-0.11</v>
+      </c>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
       <c r="I15" s="1">
         <v>32</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>10</v>
+      <c r="J15" s="1">
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="K15" s="1">
         <v>2</v>
       </c>
-      <c r="L15" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N15" s="6">
-        <v>10</v>
+      <c r="N15" s="1">
+        <v>20</v>
       </c>
       <c r="O15" s="4">
         <v>0.04</v>
@@ -1106,8 +1109,8 @@
       <c r="P15" s="3">
         <v>4.6600000000000003E-2</v>
       </c>
-      <c r="Q15" s="7">
-        <v>6.3799999999999996E-2</v>
+      <c r="Q15" s="3">
+        <v>3.9300000000000002E-2</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.35">
@@ -1151,13 +1154,10 @@
         <v>0.04</v>
       </c>
       <c r="P16" s="3">
-        <v>4.6100000000000002E-2</v>
+        <v>4.6600000000000003E-2</v>
       </c>
       <c r="Q16" s="7">
-        <v>6.3299999999999995E-2</v>
-      </c>
-      <c r="R16" t="s">
-        <v>18</v>
+        <v>6.3799999999999996E-2</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.35">
@@ -1167,35 +1167,35 @@
       <c r="B17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="1">
-        <v>0.33</v>
+      <c r="C17" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="4">
-        <v>7.0000000000000007E-2</v>
+      <c r="E17" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F17" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="5">
-        <v>0.48</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>10</v>
+        <v>0.3</v>
+      </c>
+      <c r="I17" s="1">
+        <v>32</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>10</v>
+      <c r="K17" s="1">
+        <v>2</v>
       </c>
       <c r="L17" s="8" t="s">
         <v>10</v>
       </c>
       <c r="N17" s="6">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="O17" s="4">
         <v>0.04</v>
@@ -1204,7 +1204,10 @@
         <v>4.6100000000000002E-2</v>
       </c>
       <c r="Q17" s="7">
-        <v>8.3500000000000005E-2</v>
+        <v>6.3299999999999995E-2</v>
+      </c>
+      <c r="R17" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.35">
@@ -1226,14 +1229,14 @@
       <c r="F18" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>10</v>
+      <c r="G18" s="5">
+        <v>0.48</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J18" s="1">
-        <v>2.5000000000000001E-2</v>
+      <c r="J18" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K18" s="1" t="s">
         <v>10</v>
@@ -1242,80 +1245,77 @@
         <v>10</v>
       </c>
       <c r="N18" s="6">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="O18" s="4">
         <v>0.04</v>
       </c>
       <c r="P18" s="3">
+        <v>4.6100000000000002E-2</v>
+      </c>
+      <c r="Q18" s="7">
+        <v>8.3500000000000005E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0.33</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J19" s="1">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N19" s="6">
+        <v>80</v>
+      </c>
+      <c r="O19" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="P19" s="3">
         <v>4.4400000000000002E-2</v>
       </c>
-      <c r="Q18" s="7">
+      <c r="Q19" s="7">
         <v>8.5900000000000004E-2</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R19" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-    </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C20" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L20" s="8">
-        <v>1</v>
-      </c>
-      <c r="N20">
-        <v>9</v>
-      </c>
-      <c r="O20" s="3">
-        <v>0.04</v>
-      </c>
-      <c r="P20" s="3">
-        <v>7.1599999999999997E-2</v>
-      </c>
-      <c r="Q20" s="7">
-        <v>0.08</v>
-      </c>
-      <c r="R20" t="s">
-        <v>18</v>
-      </c>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1355,13 +1355,13 @@
         <v>9</v>
       </c>
       <c r="O21" s="3">
-        <v>3.6499999999999998E-2</v>
+        <v>0.04</v>
       </c>
       <c r="P21" s="3">
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q21" s="7">
-        <v>7.9299999999999995E-2</v>
+        <v>0.08</v>
       </c>
       <c r="R21" t="s">
         <v>18</v>
@@ -1380,8 +1380,8 @@
       <c r="D22" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="4">
-        <v>0.1225</v>
+      <c r="E22" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>10</v>
@@ -1411,7 +1411,7 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q22" s="7">
-        <v>8.0500000000000002E-2</v>
+        <v>7.9299999999999995E-2</v>
       </c>
       <c r="R22" t="s">
         <v>18</v>
@@ -1442,14 +1442,14 @@
       <c r="I23" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J23" s="1">
-        <v>0.04</v>
+      <c r="J23" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L23" s="8" t="s">
-        <v>10</v>
+      <c r="L23" s="8">
+        <v>1</v>
       </c>
       <c r="N23">
         <v>9</v>
@@ -1461,72 +1461,72 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q23" s="7">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="R23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0.1225</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J24" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N24">
+        <v>9</v>
+      </c>
+      <c r="O24" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="P24" s="3">
+        <v>7.1599999999999997E-2</v>
+      </c>
+      <c r="Q24" s="7">
         <v>8.4900000000000003E-2</v>
       </c>
-      <c r="R23" t="s">
+      <c r="R24" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="N24" s="10"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="3"/>
-    </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="F25" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="1">
-        <v>2</v>
-      </c>
-      <c r="J25" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="K25" s="1">
-        <v>2</v>
-      </c>
-      <c r="L25" s="8">
-        <v>1</v>
-      </c>
-      <c r="N25" s="10">
-        <v>8</v>
-      </c>
-      <c r="O25" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="P25" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="Q25" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="R25" t="s">
-        <v>22</v>
-      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="N25" s="10"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1559,11 +1559,11 @@
       <c r="K26" s="1">
         <v>2</v>
       </c>
-      <c r="L26" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N26">
-        <v>10</v>
+      <c r="L26" s="8">
+        <v>1</v>
+      </c>
+      <c r="N26" s="10">
+        <v>8</v>
       </c>
       <c r="O26" s="3">
         <v>2.3E-2</v>
@@ -1572,141 +1572,181 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="Q26" s="7">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="R26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="1">
+        <v>2</v>
+      </c>
+      <c r="J27" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="K27" s="1">
+        <v>2</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N27">
+        <v>10</v>
+      </c>
+      <c r="O27" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="P27" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="Q27" s="7">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="R26" t="s">
+      <c r="R27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-    </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C28" s="1">
+      <c r="B29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C29" s="1">
         <v>0.125</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D29" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E29" s="4">
         <v>0.1</v>
       </c>
-      <c r="F28" s="4">
+      <c r="F29" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="G28" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L28" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N28">
-        <v>10</v>
-      </c>
-      <c r="O28" s="3">
+      <c r="G29" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N29">
+        <v>10</v>
+      </c>
+      <c r="O29" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P28" s="3">
+      <c r="P29" s="3">
         <v>0.1082</v>
       </c>
-      <c r="Q28" s="7">
+      <c r="Q29" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="R28" t="s">
+      <c r="R29" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
-    </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C30" s="1">
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1">
         <v>0.22500000000000001</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D31" s="1">
         <v>-1.6E-2</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E31" s="4">
         <v>0.18099999999999999</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K30" s="1">
+      <c r="F31" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K31" s="1">
         <v>2</v>
       </c>
-      <c r="L30" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N30">
+      <c r="L31" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N31">
         <v>27</v>
       </c>
-      <c r="O30" s="3">
+      <c r="O31" s="3">
         <v>2.3E-2</v>
       </c>
-      <c r="P30" s="3">
+      <c r="P31" s="3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="Q31" s="7">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="R30" t="s">
+      <c r="R31" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="P31" s="3"/>
-      <c r="Q31" s="3"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C32" s="1"/>
@@ -1723,6 +1763,7 @@
       <c r="D33" s="1"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
+      <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
@@ -1730,7 +1771,10 @@
     <row r="34" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
       <c r="J34" s="1"/>
+      <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
     </row>
     <row r="35" spans="3:17" x14ac:dyDescent="0.35">
@@ -1742,6 +1786,7 @@
     <row r="36" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
+      <c r="J36" s="1"/>
       <c r="Q36" s="3"/>
     </row>
     <row r="37" spans="3:17" x14ac:dyDescent="0.35">
@@ -1752,9 +1797,11 @@
     <row r="38" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
+      <c r="Q38" s="3"/>
     </row>
     <row r="39" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
     </row>
     <row r="40" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C40" s="1"/>
@@ -1764,6 +1811,9 @@
     </row>
     <row r="42" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C42" s="1"/>
+    </row>
+    <row r="43" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="C43" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Config: Discovered better CLOI factors based on testing JAAA. CLOI holds variable rate securities and is more triggered by the 2 year (short duration) changes. It is conservative and now down to 1 historical sell. JAAA had much more history.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="382" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3D1C113-8AE1-4CAC-8558-9390575B3DD9}"/>
+  <xr:revisionPtr revIDLastSave="403" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABDDF228-D47A-4ED6-B2B3-C95DB8CB2080}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="1170" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="35">
   <si>
     <t>Fund</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>updated data as of 3/20/26</t>
+  </si>
+  <si>
+    <t>Modeled after JAAA on 3/20/2026 data. Only 1 trade.</t>
   </si>
 </sst>
 </file>
@@ -545,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -1518,65 +1521,65 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="N25" s="10"/>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="3"/>
+      <c r="A25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0.17</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J25" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N25" s="10">
+        <v>1</v>
+      </c>
+      <c r="O25" s="3">
+        <v>3.6499999999999998E-2</v>
+      </c>
+      <c r="P25" s="3">
+        <v>7.1300000000000002E-2</v>
+      </c>
+      <c r="Q25" s="7">
+        <v>7.7700000000000005E-2</v>
+      </c>
+      <c r="R25" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="4">
-        <v>0.125</v>
-      </c>
-      <c r="F26" s="4">
-        <v>0.14099999999999999</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I26" s="1">
-        <v>2</v>
-      </c>
-      <c r="J26" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="K26" s="1">
-        <v>2</v>
-      </c>
-      <c r="L26" s="8">
-        <v>1</v>
-      </c>
-      <c r="N26" s="10">
-        <v>8</v>
-      </c>
-      <c r="O26" s="3">
-        <v>2.3E-2</v>
-      </c>
-      <c r="P26" s="3">
-        <v>2.1399999999999999E-2</v>
-      </c>
-      <c r="Q26" s="7">
-        <v>2.7099999999999999E-2</v>
-      </c>
-      <c r="R26" t="s">
-        <v>22</v>
-      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="N26" s="10"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
@@ -1609,11 +1612,11 @@
       <c r="K27" s="1">
         <v>2</v>
       </c>
-      <c r="L27" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N27">
-        <v>10</v>
+      <c r="L27" s="8">
+        <v>1</v>
+      </c>
+      <c r="N27" s="10">
+        <v>8</v>
       </c>
       <c r="O27" s="3">
         <v>2.3E-2</v>
@@ -1622,141 +1625,181 @@
         <v>2.1399999999999999E-2</v>
       </c>
       <c r="Q27" s="7">
+        <v>2.7099999999999999E-2</v>
+      </c>
+      <c r="R27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" s="4">
+        <v>0.125</v>
+      </c>
+      <c r="F28" s="4">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I28" s="1">
+        <v>2</v>
+      </c>
+      <c r="J28" s="1">
+        <v>2.4E-2</v>
+      </c>
+      <c r="K28" s="1">
+        <v>2</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N28">
+        <v>10</v>
+      </c>
+      <c r="O28" s="3">
+        <v>2.3E-2</v>
+      </c>
+      <c r="P28" s="3">
+        <v>2.1399999999999999E-2</v>
+      </c>
+      <c r="Q28" s="7">
         <v>2.7799999999999998E-2</v>
       </c>
-      <c r="R27" t="s">
+      <c r="R28" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-    </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C29" s="1">
+      <c r="B30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="1">
         <v>0.125</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D30" s="1">
         <v>-1.7999999999999999E-2</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E30" s="4">
         <v>0.1</v>
       </c>
-      <c r="F29" s="4">
+      <c r="F30" s="4">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="G29" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L29" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N29">
-        <v>10</v>
-      </c>
-      <c r="O29" s="3">
+      <c r="G30" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N30">
+        <v>10</v>
+      </c>
+      <c r="O30" s="3">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="P29" s="3">
+      <c r="P30" s="3">
         <v>0.1082</v>
       </c>
-      <c r="Q29" s="7">
+      <c r="Q30" s="7">
         <v>0.14130000000000001</v>
       </c>
-      <c r="R29" t="s">
+      <c r="R30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="P30" s="3"/>
-      <c r="Q30" s="3"/>
-    </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" s="1">
+      <c r="B32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C32" s="1">
         <v>0.22500000000000001</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D32" s="1">
         <v>-1.6E-2</v>
       </c>
-      <c r="E31" s="4">
+      <c r="E32" s="4">
         <v>0.18099999999999999</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K31" s="1">
+      <c r="F32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K32" s="1">
         <v>2</v>
       </c>
-      <c r="L31" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N31">
+      <c r="L32" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N32">
         <v>27</v>
       </c>
-      <c r="O31" s="3">
+      <c r="O32" s="3">
         <v>2.3E-2</v>
       </c>
-      <c r="P31" s="3">
+      <c r="P32" s="3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="Q31" s="7">
+      <c r="Q32" s="7">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="R31" t="s">
+      <c r="R32" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-      <c r="P32" s="3"/>
-      <c r="Q32" s="3"/>
     </row>
     <row r="33" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C33" s="1"/>
@@ -1773,6 +1816,7 @@
       <c r="D34" s="1"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
+      <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
@@ -1780,7 +1824,10 @@
     <row r="35" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
       <c r="J35" s="1"/>
+      <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
     </row>
     <row r="36" spans="3:17" x14ac:dyDescent="0.35">
@@ -1792,6 +1839,7 @@
     <row r="37" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
+      <c r="J37" s="1"/>
       <c r="Q37" s="3"/>
     </row>
     <row r="38" spans="3:17" x14ac:dyDescent="0.35">
@@ -1802,9 +1850,11 @@
     <row r="39" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
+      <c r="Q39" s="3"/>
     </row>
     <row r="40" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
     </row>
     <row r="41" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C41" s="1"/>
@@ -1814,6 +1864,9 @@
     </row>
     <row r="43" spans="3:17" x14ac:dyDescent="0.35">
       <c r="C43" s="1"/>
+    </row>
+    <row r="44" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="C44" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Bug Fix: Discrepancy as to how Drop was calculated in 2 different places. Config changes.
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="403" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABDDF228-D47A-4ED6-B2B3-C95DB8CB2080}"/>
+  <xr:revisionPtr revIDLastSave="417" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF7D5BCA-0557-4E82-BE90-87C002FC6261}"/>
   <bookViews>
-    <workbookView xWindow="420" yWindow="740" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="80" yWindow="720" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="37">
   <si>
     <t>Fund</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>Modeled after JAAA on 3/20/2026 data. Only 1 trade.</t>
+  </si>
+  <si>
+    <t>updated data as of 3/27/26</t>
+  </si>
+  <si>
+    <t>Lower yield but better tested. Used FAGIX for history</t>
   </si>
 </sst>
 </file>
@@ -184,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -210,6 +216,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8597F94-DE6E-4E39-917A-8E4C5B78A4E7}">
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.90625" style="1" bestFit="1" customWidth="1"/>
@@ -558,6 +565,7 @@
     <col min="12" max="12" width="11.36328125" style="8" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="11.36328125" style="8" customWidth="1"/>
     <col min="15" max="15" width="8.7265625" style="3"/>
+    <col min="19" max="19" width="9.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
@@ -1060,13 +1068,13 @@
         <v>2.3E-2</v>
       </c>
       <c r="P13" s="3">
-        <v>1.4200000000000001E-2</v>
+        <v>1.3299999999999999E-2</v>
       </c>
       <c r="Q13" s="7">
-        <v>6.1899999999999997E-2</v>
+        <v>6.59E-2</v>
       </c>
       <c r="R13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -1163,7 +1171,7 @@
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -1213,7 +1221,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -1260,7 +1268,7 @@
         <v>8.3500000000000005E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1310,7 +1318,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="4"/>
@@ -1320,7 +1328,7 @@
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1370,7 +1378,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1420,7 +1428,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -1470,7 +1478,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -1520,7 +1528,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>19</v>
       </c>
@@ -1570,7 +1578,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="4"/>
@@ -1581,7 +1589,7 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1631,7 +1639,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -1681,7 +1689,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="4"/>
@@ -1691,7 +1699,7 @@
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1741,77 +1749,123 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="P31" s="3"/>
-      <c r="Q31" s="3"/>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="1">
+        <v>-1.0999999999999999E-2</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J31" s="1">
+        <v>1E-3</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N31">
+        <v>7</v>
+      </c>
+      <c r="O31" s="3">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="P31" s="3">
+        <v>0.1009</v>
+      </c>
+      <c r="Q31" s="7">
+        <v>0.1171</v>
+      </c>
+      <c r="R31" t="s">
+        <v>24</v>
+      </c>
+      <c r="S31" s="11">
+        <v>46108</v>
+      </c>
+      <c r="T31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>28</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="1">
+      <c r="B33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="1">
         <v>0.22500000000000001</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D33" s="1">
         <v>-1.6E-2</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E33" s="4">
         <v>0.18099999999999999</v>
       </c>
-      <c r="F32" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K32" s="1">
+      <c r="F33" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K33" s="1">
         <v>2</v>
       </c>
-      <c r="L32" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N32">
+      <c r="L33" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="N33">
         <v>27</v>
       </c>
-      <c r="O32" s="3">
+      <c r="O33" s="3">
         <v>2.3E-2</v>
       </c>
-      <c r="P32" s="3">
+      <c r="P33" s="3">
         <v>4.3499999999999997E-2</v>
       </c>
-      <c r="Q32" s="7">
+      <c r="Q33" s="7">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="R32" t="s">
+      <c r="R33" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="3:17" x14ac:dyDescent="0.35">
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="P33" s="3"/>
-      <c r="Q33" s="3"/>
-    </row>
-    <row r="34" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
       <c r="E34" s="4"/>
@@ -1821,52 +1875,62 @@
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
     </row>
-    <row r="35" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
+      <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
     </row>
-    <row r="36" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
       <c r="J36" s="1"/>
+      <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
     </row>
-    <row r="37" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="J37" s="1"/>
       <c r="Q37" s="3"/>
     </row>
-    <row r="38" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
+      <c r="J38" s="1"/>
       <c r="Q38" s="3"/>
     </row>
-    <row r="39" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="Q39" s="3"/>
     </row>
-    <row r="40" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
-    </row>
-    <row r="41" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="Q40" s="3"/>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C41" s="1"/>
-    </row>
-    <row r="42" spans="3:17" x14ac:dyDescent="0.35">
+      <c r="D41" s="1"/>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C42" s="1"/>
     </row>
-    <row r="43" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C43" s="1"/>
     </row>
-    <row r="44" spans="3:17" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C44" s="1"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="C45" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Config: Updated data files
</commit_message>
<xml_diff>
--- a/FundOptimizationResults.xlsx
+++ b/FundOptimizationResults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dd266ef2451b5a0b/Documents/Finance/strat-opt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="417" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF7D5BCA-0557-4E82-BE90-87C002FC6261}"/>
+  <xr:revisionPtr revIDLastSave="438" documentId="8_{30E8992D-C6A0-4761-AFEB-3D1BCFD7E691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{07580A55-8EDB-49DB-9185-03704ED38A7A}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="720" windowWidth="25180" windowHeight="15260" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
+    <workbookView xWindow="2660" yWindow="1570" windowWidth="21740" windowHeight="14430" xr2:uid="{438A0D2B-B48C-423F-9128-A2BAAC94AEB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="36">
   <si>
     <t>Fund</t>
   </si>
@@ -113,9 +113,6 @@
     <t>data as of 3/11/26</t>
   </si>
   <si>
-    <t>Use drop instead of delta yield 10</t>
-  </si>
-  <si>
     <t>data as of 3/9/26</t>
   </si>
   <si>
@@ -140,13 +137,13 @@
     <t>updated data as of 3/20/26</t>
   </si>
   <si>
-    <t>Modeled after JAAA on 3/20/2026 data. Only 1 trade.</t>
-  </si>
-  <si>
     <t>updated data as of 3/27/26</t>
   </si>
   <si>
     <t>Lower yield but better tested. Used FAGIX for history</t>
+  </si>
+  <si>
+    <t>updated as of 4/17/26</t>
   </si>
 </sst>
 </file>
@@ -570,10 +567,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="C1" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="10" t="s">
         <v>30</v>
-      </c>
-      <c r="J1" s="10" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:18" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -793,7 +790,7 @@
         <v>6.5199999999999994E-2</v>
       </c>
       <c r="R6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
@@ -843,7 +840,7 @@
         <v>7.4099999999999999E-2</v>
       </c>
       <c r="R7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
@@ -1024,7 +1021,7 @@
         <v>5.79E-2</v>
       </c>
       <c r="R12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.35">
@@ -1074,7 +1071,7 @@
         <v>6.59E-2</v>
       </c>
       <c r="R13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.35">
@@ -1315,7 +1312,7 @@
         <v>8.5900000000000004E-2</v>
       </c>
       <c r="R19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.35">
@@ -1472,7 +1469,7 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q23" s="7">
-        <v>8.0500000000000002E-2</v>
+        <v>8.3299999999999999E-2</v>
       </c>
       <c r="R23" t="s">
         <v>18</v>
@@ -1485,17 +1482,17 @@
       <c r="B24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="1">
-        <v>0.1</v>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E24" s="4">
-        <v>0.1225</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>10</v>
+      <c r="E24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0.16500000000000001</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>10</v>
@@ -1503,17 +1500,17 @@
       <c r="I24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J24" s="1">
-        <v>0.04</v>
+      <c r="J24" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L24" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N24">
-        <v>9</v>
+      <c r="L24" s="8">
+        <v>1</v>
+      </c>
+      <c r="N24" s="10">
+        <v>1</v>
       </c>
       <c r="O24" s="3">
         <v>3.6499999999999998E-2</v>
@@ -1522,61 +1519,21 @@
         <v>7.1599999999999997E-2</v>
       </c>
       <c r="Q24" s="7">
-        <v>8.4900000000000003E-2</v>
+        <v>8.1500000000000003E-2</v>
       </c>
       <c r="R24" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" s="4">
-        <v>0.17</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J25" s="1">
-        <v>2.4E-2</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L25" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="N25" s="10">
-        <v>1</v>
-      </c>
-      <c r="O25" s="3">
-        <v>3.6499999999999998E-2</v>
-      </c>
-      <c r="P25" s="3">
-        <v>7.1300000000000002E-2</v>
-      </c>
-      <c r="Q25" s="7">
-        <v>7.7700000000000005E-2</v>
-      </c>
-      <c r="R25" t="s">
-        <v>34</v>
-      </c>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="7"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="C26" s="1"/>
@@ -1686,7 +1643,7 @@
         <v>2.7799999999999998E-2</v>
       </c>
       <c r="R28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.35">
@@ -1802,7 +1759,7 @@
         <v>46108</v>
       </c>
       <c r="T31" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.35">
@@ -1817,7 +1774,7 @@
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>10</v>
@@ -1862,7 +1819,7 @@
         <v>6.4500000000000002E-2</v>
       </c>
       <c r="R33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.35">

</xml_diff>